<commit_message>
update Huawei materials with company info
</commit_message>
<xml_diff>
--- a/huawei/huawei-health-application-draft-2026-10-15.xlsx
+++ b/huawei/huawei-health-application-draft-2026-10-15.xlsx
@@ -530,7 +530,6 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
@@ -580,14 +579,14 @@
           <t>企业全称</t>
         </is>
       </c>
-      <c r="B2" s="6" t="inlineStr">
-        <is>
-          <t>[营业执照上的公司全称]</t>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>北京小巢科技有限公司</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>树补充</t>
+          <t>树 10/15 提供</t>
         </is>
       </c>
     </row>
@@ -614,14 +613,14 @@
           <t>成立日期</t>
         </is>
       </c>
-      <c r="B4" s="6" t="inlineStr">
-        <is>
-          <t>[YYYY-MM-DD]</t>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>2018-11-27</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>华为要求企业主体成立满 1 年</t>
+          <t>树 10/15 提供；满足「成立 ≥ 1 年」</t>
         </is>
       </c>
     </row>
@@ -650,12 +649,12 @@
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>[地址]</t>
+          <t>北京市（详细地址以营业执照为准）</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>树补充</t>
+          <t>树提供到城市；模板若要求详细地址请按营业执照补</t>
         </is>
       </c>
     </row>
@@ -1459,14 +1458,14 @@
           <t>业务联系人</t>
         </is>
       </c>
-      <c r="B2" s="6" t="inlineStr">
-        <is>
-          <t>[姓名]</t>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>张树</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>树补充</t>
+          <t>树 10/15 提供</t>
         </is>
       </c>
     </row>
@@ -1478,12 +1477,12 @@
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>[手机号]</t>
+          <t>（请在华为申请表里直接填写）</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>树补充</t>
+          <t>手机号不放进公开文件</t>
         </is>
       </c>
     </row>

</xml_diff>